<commit_message>
Improve again Loan menu
</commit_message>
<xml_diff>
--- a/Permissions.xlsx
+++ b/Permissions.xlsx
@@ -1,10 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
-  <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
-  <workbookPr defaultThemeVersion="164011"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30228"/>
+  <workbookPr/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Erfan\source\repos\LibraryManagementSystem\"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{35343F2B-5A7C-4C00-9B38-C38A68B6B949}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="22260" windowHeight="12645"/>
+    <workbookView xWindow="-105" yWindow="0" windowWidth="14325" windowHeight="16305" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -18,15 +24,213 @@
 </workbook>
 </file>
 
+<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="59" uniqueCount="39">
+  <si>
+    <t>Permissions</t>
+  </si>
+  <si>
+    <t>Admin</t>
+  </si>
+  <si>
+    <t>Librarian</t>
+  </si>
+  <si>
+    <t>Member</t>
+  </si>
+  <si>
+    <t>Top Menu</t>
+  </si>
+  <si>
+    <t>Authors</t>
+  </si>
+  <si>
+    <t>Translators</t>
+  </si>
+  <si>
+    <t>Books</t>
+  </si>
+  <si>
+    <t>Members</t>
+  </si>
+  <si>
+    <t>Loans</t>
+  </si>
+  <si>
+    <t>Fines</t>
+  </si>
+  <si>
+    <t>Logout</t>
+  </si>
+  <si>
+    <t>Add</t>
+  </si>
+  <si>
+    <t>Edit</t>
+  </si>
+  <si>
+    <t>Remove</t>
+  </si>
+  <si>
+    <t>Search</t>
+  </si>
+  <si>
+    <t>View Detail</t>
+  </si>
+  <si>
+    <t>View All</t>
+  </si>
+  <si>
+    <t>Change Password</t>
+  </si>
+  <si>
+    <t>Borrow Book</t>
+  </si>
+  <si>
+    <t>Return Book</t>
+  </si>
+  <si>
+    <t>Renew Book</t>
+  </si>
+  <si>
+    <t>My Active Loans</t>
+  </si>
+  <si>
+    <t>Active Loans By User</t>
+  </si>
+  <si>
+    <t>Active Loans By Book</t>
+  </si>
+  <si>
+    <t>My Overdue Loans</t>
+  </si>
+  <si>
+    <t>OverDue Loans By User</t>
+  </si>
+  <si>
+    <t>History By Book</t>
+  </si>
+  <si>
+    <t>History By User</t>
+  </si>
+  <si>
+    <t>Full Library History</t>
+  </si>
+  <si>
+    <t>Pay Fine</t>
+  </si>
+  <si>
+    <t>Waive Fine</t>
+  </si>
+  <si>
+    <t>View Fines By User</t>
+  </si>
+  <si>
+    <t>View Fines By Book</t>
+  </si>
+  <si>
+    <t>View Unpaid Fines By User</t>
+  </si>
+  <si>
+    <t>My Unpaid Fines</t>
+  </si>
+  <si>
+    <t>My Fines</t>
+  </si>
+  <si>
+    <t>View Unpaid Fines By Book</t>
+  </si>
+  <si>
+    <t>History Of Fines</t>
+  </si>
+</sst>
+</file>
+
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
-  <fonts count="1" x14ac:knownFonts="1">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <fonts count="13" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="16"/>
+      <color theme="1"/>
+      <name val="JetBrains Mono Medium"/>
+      <family val="3"/>
+    </font>
+    <font>
+      <sz val="16"/>
+      <color rgb="FFC00000"/>
+      <name val="JetBrains Mono Medium"/>
+      <family val="3"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FFC00000"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="16"/>
+      <color rgb="FFFFC000"/>
+      <name val="JetBrains Mono Medium"/>
+      <family val="3"/>
+    </font>
+    <font>
+      <sz val="16"/>
+      <color rgb="FF92D050"/>
+      <name val="JetBrains Mono Medium"/>
+      <family val="3"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF92D050"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="16"/>
+      <color rgb="FF00B0F0"/>
+      <name val="JetBrains Mono Medium"/>
+      <family val="3"/>
+    </font>
+    <font>
+      <sz val="16"/>
+      <color rgb="FF00B050"/>
+      <name val="JetBrains Mono Medium"/>
+      <family val="3"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF00B050"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="16"/>
+      <color rgb="FF7030A0"/>
+      <name val="JetBrains Mono Medium"/>
+      <family val="3"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF7030A0"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="16"/>
+      <color rgb="FF0070C0"/>
+      <name val="JetBrains Mono Medium"/>
+      <family val="3"/>
     </font>
   </fonts>
   <fills count="2">
@@ -49,8 +253,20 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="13">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -330,10 +546,578 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+  <dimension ref="A1:G49"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
-  <sheetData/>
+  <cols>
+    <col min="1" max="1" width="25.140625" customWidth="1"/>
+    <col min="2" max="2" width="48" customWidth="1"/>
+    <col min="3" max="3" width="11.5703125" customWidth="1"/>
+    <col min="4" max="4" width="19.42578125" customWidth="1"/>
+    <col min="5" max="5" width="14.28515625" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:7" ht="21" x14ac:dyDescent="0.35">
+      <c r="A1" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="F1" s="1"/>
+      <c r="G1" s="1"/>
+    </row>
+    <row r="2" spans="1:7" ht="21" x14ac:dyDescent="0.35">
+      <c r="A2" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="B2" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="C2" s="2"/>
+      <c r="D2" s="2"/>
+      <c r="E2" s="2"/>
+      <c r="F2" s="1"/>
+      <c r="G2" s="1"/>
+    </row>
+    <row r="3" spans="1:7" ht="21" x14ac:dyDescent="0.35">
+      <c r="A3" s="2"/>
+      <c r="B3" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="C3" s="2"/>
+      <c r="D3" s="2"/>
+      <c r="E3" s="2"/>
+      <c r="F3" s="1"/>
+      <c r="G3" s="1"/>
+    </row>
+    <row r="4" spans="1:7" ht="21" x14ac:dyDescent="0.35">
+      <c r="A4" s="2"/>
+      <c r="B4" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="C4" s="2"/>
+      <c r="D4" s="2"/>
+      <c r="E4" s="2"/>
+      <c r="F4" s="1"/>
+      <c r="G4" s="1"/>
+    </row>
+    <row r="5" spans="1:7" ht="21" x14ac:dyDescent="0.35">
+      <c r="A5" s="2"/>
+      <c r="B5" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="C5" s="2"/>
+      <c r="D5" s="2"/>
+      <c r="E5" s="2"/>
+      <c r="F5" s="1"/>
+      <c r="G5" s="1"/>
+    </row>
+    <row r="6" spans="1:7" ht="21" x14ac:dyDescent="0.35">
+      <c r="A6" s="2"/>
+      <c r="B6" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="C6" s="2"/>
+      <c r="D6" s="2"/>
+      <c r="E6" s="2"/>
+      <c r="F6" s="1"/>
+      <c r="G6" s="1"/>
+    </row>
+    <row r="7" spans="1:7" ht="21" x14ac:dyDescent="0.35">
+      <c r="A7" s="3"/>
+      <c r="B7" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="C7" s="2"/>
+      <c r="D7" s="2"/>
+      <c r="E7" s="2"/>
+      <c r="F7" s="1"/>
+      <c r="G7" s="1"/>
+    </row>
+    <row r="8" spans="1:7" ht="21" x14ac:dyDescent="0.35">
+      <c r="A8" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="B8" s="4" t="s">
+        <v>12</v>
+      </c>
+      <c r="C8" s="4"/>
+      <c r="D8" s="4"/>
+      <c r="E8" s="4"/>
+      <c r="F8" s="1"/>
+      <c r="G8" s="1"/>
+    </row>
+    <row r="9" spans="1:7" ht="21" x14ac:dyDescent="0.35">
+      <c r="A9" s="4"/>
+      <c r="B9" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="C9" s="4"/>
+      <c r="D9" s="4"/>
+      <c r="E9" s="4"/>
+      <c r="F9" s="1"/>
+      <c r="G9" s="1"/>
+    </row>
+    <row r="10" spans="1:7" ht="21" x14ac:dyDescent="0.35">
+      <c r="A10" s="4"/>
+      <c r="B10" s="4" t="s">
+        <v>14</v>
+      </c>
+      <c r="C10" s="4"/>
+      <c r="D10" s="4"/>
+      <c r="E10" s="4"/>
+      <c r="F10" s="1"/>
+      <c r="G10" s="1"/>
+    </row>
+    <row r="11" spans="1:7" ht="21" x14ac:dyDescent="0.35">
+      <c r="A11" s="4"/>
+      <c r="B11" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="C11" s="4"/>
+      <c r="D11" s="4"/>
+      <c r="E11" s="4"/>
+      <c r="F11" s="1"/>
+      <c r="G11" s="1"/>
+    </row>
+    <row r="12" spans="1:7" ht="21" x14ac:dyDescent="0.35">
+      <c r="A12" s="4"/>
+      <c r="B12" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="C12" s="4"/>
+      <c r="D12" s="4"/>
+      <c r="E12" s="4"/>
+      <c r="F12" s="1"/>
+      <c r="G12" s="1"/>
+    </row>
+    <row r="13" spans="1:7" ht="21" x14ac:dyDescent="0.35">
+      <c r="A13" s="4"/>
+      <c r="B13" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="C13" s="4"/>
+      <c r="D13" s="4"/>
+      <c r="E13" s="4"/>
+      <c r="F13" s="1"/>
+      <c r="G13" s="1"/>
+    </row>
+    <row r="14" spans="1:7" ht="21" x14ac:dyDescent="0.35">
+      <c r="A14" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="B14" s="5" t="s">
+        <v>12</v>
+      </c>
+      <c r="C14" s="5"/>
+      <c r="D14" s="5"/>
+      <c r="E14" s="5"/>
+      <c r="F14" s="1"/>
+      <c r="G14" s="1"/>
+    </row>
+    <row r="15" spans="1:7" ht="21" x14ac:dyDescent="0.35">
+      <c r="A15" s="6"/>
+      <c r="B15" s="5" t="s">
+        <v>13</v>
+      </c>
+      <c r="C15" s="5"/>
+      <c r="D15" s="5"/>
+      <c r="E15" s="5"/>
+      <c r="F15" s="1"/>
+      <c r="G15" s="1"/>
+    </row>
+    <row r="16" spans="1:7" ht="21" x14ac:dyDescent="0.35">
+      <c r="A16" s="5"/>
+      <c r="B16" s="5" t="s">
+        <v>14</v>
+      </c>
+      <c r="C16" s="5"/>
+      <c r="D16" s="5"/>
+      <c r="E16" s="5"/>
+      <c r="F16" s="1"/>
+      <c r="G16" s="1"/>
+    </row>
+    <row r="17" spans="1:7" ht="21" x14ac:dyDescent="0.35">
+      <c r="A17" s="5"/>
+      <c r="B17" s="5" t="s">
+        <v>15</v>
+      </c>
+      <c r="C17" s="5"/>
+      <c r="D17" s="5"/>
+      <c r="E17" s="5"/>
+      <c r="F17" s="1"/>
+      <c r="G17" s="1"/>
+    </row>
+    <row r="18" spans="1:7" ht="21" x14ac:dyDescent="0.35">
+      <c r="A18" s="5"/>
+      <c r="B18" s="5" t="s">
+        <v>16</v>
+      </c>
+      <c r="C18" s="5"/>
+      <c r="D18" s="5"/>
+      <c r="E18" s="5"/>
+      <c r="F18" s="1"/>
+      <c r="G18" s="1"/>
+    </row>
+    <row r="19" spans="1:7" ht="21" x14ac:dyDescent="0.35">
+      <c r="A19" s="5"/>
+      <c r="B19" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="C19" s="5"/>
+      <c r="D19" s="5"/>
+      <c r="E19" s="5"/>
+      <c r="F19" s="1"/>
+      <c r="G19" s="1"/>
+    </row>
+    <row r="20" spans="1:7" ht="21" x14ac:dyDescent="0.35">
+      <c r="A20" s="7" t="s">
+        <v>8</v>
+      </c>
+      <c r="B20" s="7" t="s">
+        <v>12</v>
+      </c>
+      <c r="C20" s="7"/>
+      <c r="D20" s="7"/>
+      <c r="E20" s="7"/>
+      <c r="F20" s="1"/>
+      <c r="G20" s="1"/>
+    </row>
+    <row r="21" spans="1:7" ht="21" x14ac:dyDescent="0.35">
+      <c r="A21" s="7"/>
+      <c r="B21" s="7" t="s">
+        <v>13</v>
+      </c>
+      <c r="C21" s="7"/>
+      <c r="D21" s="7"/>
+      <c r="E21" s="7"/>
+      <c r="F21" s="1"/>
+      <c r="G21" s="1"/>
+    </row>
+    <row r="22" spans="1:7" ht="21" x14ac:dyDescent="0.35">
+      <c r="A22" s="7"/>
+      <c r="B22" s="7" t="s">
+        <v>14</v>
+      </c>
+      <c r="C22" s="7"/>
+      <c r="D22" s="7"/>
+      <c r="E22" s="7"/>
+      <c r="F22" s="1"/>
+      <c r="G22" s="1"/>
+    </row>
+    <row r="23" spans="1:7" ht="21" x14ac:dyDescent="0.35">
+      <c r="A23" s="7"/>
+      <c r="B23" s="7" t="s">
+        <v>15</v>
+      </c>
+      <c r="C23" s="7"/>
+      <c r="D23" s="7"/>
+      <c r="E23" s="7"/>
+      <c r="F23" s="1"/>
+      <c r="G23" s="1"/>
+    </row>
+    <row r="24" spans="1:7" ht="21" x14ac:dyDescent="0.35">
+      <c r="A24" s="7"/>
+      <c r="B24" s="7" t="s">
+        <v>16</v>
+      </c>
+      <c r="C24" s="7"/>
+      <c r="D24" s="7"/>
+      <c r="E24" s="7"/>
+      <c r="F24" s="1"/>
+      <c r="G24" s="1"/>
+    </row>
+    <row r="25" spans="1:7" ht="21" x14ac:dyDescent="0.35">
+      <c r="A25" s="7"/>
+      <c r="B25" s="7" t="s">
+        <v>17</v>
+      </c>
+      <c r="C25" s="7"/>
+      <c r="D25" s="7"/>
+      <c r="E25" s="7"/>
+      <c r="F25" s="1"/>
+      <c r="G25" s="1"/>
+    </row>
+    <row r="26" spans="1:7" ht="21" x14ac:dyDescent="0.35">
+      <c r="A26" s="7"/>
+      <c r="B26" s="7" t="s">
+        <v>18</v>
+      </c>
+      <c r="C26" s="7"/>
+      <c r="D26" s="7"/>
+      <c r="E26" s="7"/>
+      <c r="F26" s="1"/>
+      <c r="G26" s="1"/>
+    </row>
+    <row r="27" spans="1:7" ht="21" x14ac:dyDescent="0.35">
+      <c r="A27" s="8" t="s">
+        <v>9</v>
+      </c>
+      <c r="B27" s="8" t="s">
+        <v>19</v>
+      </c>
+      <c r="C27" s="8"/>
+      <c r="D27" s="8"/>
+      <c r="E27" s="8"/>
+      <c r="F27" s="1"/>
+      <c r="G27" s="1"/>
+    </row>
+    <row r="28" spans="1:7" ht="21" x14ac:dyDescent="0.35">
+      <c r="A28" s="8"/>
+      <c r="B28" s="8" t="s">
+        <v>20</v>
+      </c>
+      <c r="C28" s="8"/>
+      <c r="D28" s="8"/>
+      <c r="E28" s="8"/>
+      <c r="F28" s="1"/>
+      <c r="G28" s="1"/>
+    </row>
+    <row r="29" spans="1:7" ht="21" x14ac:dyDescent="0.35">
+      <c r="A29" s="8"/>
+      <c r="B29" s="8" t="s">
+        <v>21</v>
+      </c>
+      <c r="C29" s="8"/>
+      <c r="D29" s="8"/>
+      <c r="E29" s="8"/>
+      <c r="F29" s="1"/>
+      <c r="G29" s="1"/>
+    </row>
+    <row r="30" spans="1:7" ht="21" x14ac:dyDescent="0.35">
+      <c r="A30" s="8"/>
+      <c r="B30" s="8" t="s">
+        <v>22</v>
+      </c>
+      <c r="C30" s="8"/>
+      <c r="D30" s="8"/>
+      <c r="E30" s="8"/>
+      <c r="F30" s="1"/>
+      <c r="G30" s="1"/>
+    </row>
+    <row r="31" spans="1:7" ht="21" x14ac:dyDescent="0.35">
+      <c r="A31" s="8"/>
+      <c r="B31" s="8" t="s">
+        <v>23</v>
+      </c>
+      <c r="C31" s="8"/>
+      <c r="D31" s="8"/>
+      <c r="E31" s="8"/>
+      <c r="F31" s="1"/>
+      <c r="G31" s="1"/>
+    </row>
+    <row r="32" spans="1:7" ht="21" x14ac:dyDescent="0.35">
+      <c r="A32" s="8"/>
+      <c r="B32" s="8" t="s">
+        <v>24</v>
+      </c>
+      <c r="C32" s="8"/>
+      <c r="D32" s="8"/>
+      <c r="E32" s="8"/>
+      <c r="F32" s="1"/>
+      <c r="G32" s="1"/>
+    </row>
+    <row r="33" spans="1:7" ht="21" x14ac:dyDescent="0.35">
+      <c r="A33" s="8"/>
+      <c r="B33" s="8" t="s">
+        <v>25</v>
+      </c>
+      <c r="C33" s="8"/>
+      <c r="D33" s="8"/>
+      <c r="E33" s="8"/>
+      <c r="F33" s="1"/>
+      <c r="G33" s="1"/>
+    </row>
+    <row r="34" spans="1:7" ht="21" x14ac:dyDescent="0.35">
+      <c r="A34" s="8"/>
+      <c r="B34" s="8" t="s">
+        <v>26</v>
+      </c>
+      <c r="C34" s="8"/>
+      <c r="D34" s="8"/>
+      <c r="E34" s="8"/>
+      <c r="F34" s="1"/>
+      <c r="G34" s="1"/>
+    </row>
+    <row r="35" spans="1:7" ht="21" x14ac:dyDescent="0.35">
+      <c r="A35" s="8"/>
+      <c r="B35" s="8" t="s">
+        <v>28</v>
+      </c>
+      <c r="C35" s="8"/>
+      <c r="D35" s="8"/>
+      <c r="E35" s="8"/>
+      <c r="F35" s="1"/>
+      <c r="G35" s="1"/>
+    </row>
+    <row r="36" spans="1:7" ht="21" x14ac:dyDescent="0.35">
+      <c r="A36" s="8"/>
+      <c r="B36" s="8" t="s">
+        <v>27</v>
+      </c>
+      <c r="C36" s="8"/>
+      <c r="D36" s="8"/>
+      <c r="E36" s="8"/>
+      <c r="F36" s="1"/>
+      <c r="G36" s="1"/>
+    </row>
+    <row r="37" spans="1:7" ht="21" x14ac:dyDescent="0.35">
+      <c r="A37" s="9"/>
+      <c r="B37" s="8" t="s">
+        <v>29</v>
+      </c>
+      <c r="C37" s="8"/>
+      <c r="D37" s="8"/>
+      <c r="E37" s="8"/>
+      <c r="F37" s="1"/>
+      <c r="G37" s="1"/>
+    </row>
+    <row r="38" spans="1:7" ht="21" x14ac:dyDescent="0.35">
+      <c r="A38" s="8"/>
+      <c r="B38" s="8" t="s">
+        <v>15</v>
+      </c>
+      <c r="C38" s="8"/>
+      <c r="D38" s="8"/>
+      <c r="E38" s="8"/>
+      <c r="F38" s="1"/>
+      <c r="G38" s="1"/>
+    </row>
+    <row r="39" spans="1:7" ht="21" x14ac:dyDescent="0.35">
+      <c r="A39" s="10" t="s">
+        <v>10</v>
+      </c>
+      <c r="B39" s="10" t="s">
+        <v>30</v>
+      </c>
+      <c r="C39" s="10"/>
+      <c r="D39" s="10"/>
+      <c r="E39" s="10"/>
+      <c r="F39" s="1"/>
+      <c r="G39" s="1"/>
+    </row>
+    <row r="40" spans="1:7" ht="21" x14ac:dyDescent="0.35">
+      <c r="A40" s="10"/>
+      <c r="B40" s="10" t="s">
+        <v>31</v>
+      </c>
+      <c r="C40" s="10"/>
+      <c r="D40" s="10"/>
+      <c r="E40" s="10"/>
+      <c r="F40" s="1"/>
+      <c r="G40" s="1"/>
+    </row>
+    <row r="41" spans="1:7" ht="21" x14ac:dyDescent="0.35">
+      <c r="A41" s="10"/>
+      <c r="B41" s="10" t="s">
+        <v>36</v>
+      </c>
+      <c r="C41" s="10"/>
+      <c r="D41" s="10"/>
+      <c r="E41" s="10"/>
+      <c r="F41" s="1"/>
+      <c r="G41" s="1"/>
+    </row>
+    <row r="42" spans="1:7" ht="21" x14ac:dyDescent="0.35">
+      <c r="A42" s="10"/>
+      <c r="B42" s="10" t="s">
+        <v>32</v>
+      </c>
+      <c r="C42" s="10"/>
+      <c r="D42" s="10"/>
+      <c r="E42" s="10"/>
+      <c r="F42" s="1"/>
+      <c r="G42" s="1"/>
+    </row>
+    <row r="43" spans="1:7" ht="21" x14ac:dyDescent="0.35">
+      <c r="A43" s="10"/>
+      <c r="B43" s="10" t="s">
+        <v>33</v>
+      </c>
+      <c r="C43" s="10"/>
+      <c r="D43" s="10"/>
+      <c r="E43" s="10"/>
+      <c r="F43" s="1"/>
+      <c r="G43" s="1"/>
+    </row>
+    <row r="44" spans="1:7" ht="21" x14ac:dyDescent="0.35">
+      <c r="A44" s="11"/>
+      <c r="B44" s="10" t="s">
+        <v>35</v>
+      </c>
+      <c r="C44" s="10"/>
+      <c r="D44" s="10"/>
+      <c r="E44" s="10"/>
+      <c r="F44" s="1"/>
+      <c r="G44" s="1"/>
+    </row>
+    <row r="45" spans="1:7" ht="21" x14ac:dyDescent="0.35">
+      <c r="A45" s="10"/>
+      <c r="B45" s="10" t="s">
+        <v>34</v>
+      </c>
+      <c r="C45" s="10"/>
+      <c r="D45" s="10"/>
+      <c r="E45" s="10"/>
+      <c r="F45" s="1"/>
+      <c r="G45" s="1"/>
+    </row>
+    <row r="46" spans="1:7" ht="21" x14ac:dyDescent="0.35">
+      <c r="A46" s="10"/>
+      <c r="B46" s="10" t="s">
+        <v>37</v>
+      </c>
+      <c r="C46" s="10"/>
+      <c r="D46" s="10"/>
+      <c r="E46" s="10"/>
+      <c r="F46" s="1"/>
+      <c r="G46" s="1"/>
+    </row>
+    <row r="47" spans="1:7" ht="21" x14ac:dyDescent="0.35">
+      <c r="A47" s="10"/>
+      <c r="B47" s="10" t="s">
+        <v>38</v>
+      </c>
+      <c r="C47" s="10"/>
+      <c r="D47" s="10"/>
+      <c r="E47" s="10"/>
+      <c r="F47" s="1"/>
+      <c r="G47" s="1"/>
+    </row>
+    <row r="48" spans="1:7" ht="21" x14ac:dyDescent="0.35">
+      <c r="A48" s="12" t="s">
+        <v>11</v>
+      </c>
+      <c r="B48" s="12" t="s">
+        <v>11</v>
+      </c>
+      <c r="C48" s="12"/>
+      <c r="D48" s="12"/>
+      <c r="E48" s="12"/>
+      <c r="F48" s="1"/>
+      <c r="G48" s="1"/>
+    </row>
+    <row r="49" spans="1:7" ht="21" x14ac:dyDescent="0.35">
+      <c r="A49" s="1"/>
+      <c r="B49" s="1"/>
+      <c r="C49" s="1"/>
+      <c r="D49" s="1"/>
+      <c r="E49" s="1"/>
+      <c r="F49" s="1"/>
+      <c r="G49" s="1"/>
+    </row>
+  </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" horizontalDpi="1200" verticalDpi="1200" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Improve fine menu based on new authorization
</commit_message>
<xml_diff>
--- a/Permissions.xlsx
+++ b/Permissions.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Erfan\source\repos\LibraryManagementSystem\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{35343F2B-5A7C-4C00-9B38-C38A68B6B949}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FBF5E708-93C7-4A50-8C35-D8D0E760DAFC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-105" yWindow="0" windowWidth="14325" windowHeight="16305" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="59" uniqueCount="39">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="133" uniqueCount="43">
   <si>
     <t>Permissions</t>
   </si>
@@ -142,6 +142,18 @@
   </si>
   <si>
     <t>History Of Fines</t>
+  </si>
+  <si>
+    <t>*</t>
+  </si>
+  <si>
+    <t>Librarian can add only member, but Admin can add both.</t>
+  </si>
+  <si>
+    <t>**</t>
+  </si>
+  <si>
+    <t>Librarian can remove only member, but Admin can remove both.</t>
   </si>
 </sst>
 </file>
@@ -253,20 +265,55 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="13">
+  <cellXfs count="22">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -550,569 +597,717 @@
   <dimension ref="A1:G49"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="25.140625" customWidth="1"/>
+    <col min="1" max="1" width="21.7109375" style="17" customWidth="1"/>
     <col min="2" max="2" width="48" customWidth="1"/>
-    <col min="3" max="3" width="11.5703125" customWidth="1"/>
-    <col min="4" max="4" width="19.42578125" customWidth="1"/>
-    <col min="5" max="5" width="14.28515625" customWidth="1"/>
+    <col min="3" max="3" width="11.5703125" style="17" customWidth="1"/>
+    <col min="4" max="4" width="19.42578125" style="17" customWidth="1"/>
+    <col min="5" max="5" width="14.28515625" style="17" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:7" ht="21" x14ac:dyDescent="0.35">
-      <c r="A1" s="1" t="s">
+      <c r="A1" s="9" t="s">
         <v>4</v>
       </c>
       <c r="B1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" s="9" t="s">
         <v>1</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" s="9" t="s">
         <v>2</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" s="9" t="s">
         <v>3</v>
       </c>
       <c r="F1" s="1"/>
       <c r="G1" s="1"/>
     </row>
     <row r="2" spans="1:7" ht="21" x14ac:dyDescent="0.35">
-      <c r="A2" s="2" t="s">
+      <c r="A2" s="10" t="s">
         <v>5</v>
       </c>
       <c r="B2" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="C2" s="2"/>
-      <c r="D2" s="2"/>
-      <c r="E2" s="2"/>
+      <c r="C2" s="10" t="s">
+        <v>39</v>
+      </c>
+      <c r="D2" s="10" t="s">
+        <v>39</v>
+      </c>
+      <c r="E2" s="10"/>
       <c r="F2" s="1"/>
       <c r="G2" s="1"/>
     </row>
     <row r="3" spans="1:7" ht="21" x14ac:dyDescent="0.35">
-      <c r="A3" s="2"/>
+      <c r="A3" s="10"/>
       <c r="B3" s="2" t="s">
         <v>13</v>
       </c>
-      <c r="C3" s="2"/>
-      <c r="D3" s="2"/>
-      <c r="E3" s="2"/>
+      <c r="C3" s="10" t="s">
+        <v>39</v>
+      </c>
+      <c r="D3" s="10" t="s">
+        <v>39</v>
+      </c>
+      <c r="E3" s="10"/>
       <c r="F3" s="1"/>
       <c r="G3" s="1"/>
     </row>
     <row r="4" spans="1:7" ht="21" x14ac:dyDescent="0.35">
-      <c r="A4" s="2"/>
+      <c r="A4" s="10"/>
       <c r="B4" s="2" t="s">
         <v>14</v>
       </c>
-      <c r="C4" s="2"/>
-      <c r="D4" s="2"/>
-      <c r="E4" s="2"/>
+      <c r="C4" s="10" t="s">
+        <v>39</v>
+      </c>
+      <c r="D4" s="10"/>
+      <c r="E4" s="10"/>
       <c r="F4" s="1"/>
       <c r="G4" s="1"/>
     </row>
     <row r="5" spans="1:7" ht="21" x14ac:dyDescent="0.35">
-      <c r="A5" s="2"/>
+      <c r="A5" s="10"/>
       <c r="B5" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="C5" s="2"/>
-      <c r="D5" s="2"/>
-      <c r="E5" s="2"/>
+      <c r="C5" s="10" t="s">
+        <v>39</v>
+      </c>
+      <c r="D5" s="10" t="s">
+        <v>39</v>
+      </c>
+      <c r="E5" s="10" t="s">
+        <v>39</v>
+      </c>
       <c r="F5" s="1"/>
       <c r="G5" s="1"/>
     </row>
     <row r="6" spans="1:7" ht="21" x14ac:dyDescent="0.35">
-      <c r="A6" s="2"/>
+      <c r="A6" s="10"/>
       <c r="B6" s="2" t="s">
         <v>16</v>
       </c>
-      <c r="C6" s="2"/>
-      <c r="D6" s="2"/>
-      <c r="E6" s="2"/>
+      <c r="C6" s="10" t="s">
+        <v>39</v>
+      </c>
+      <c r="D6" s="10" t="s">
+        <v>39</v>
+      </c>
+      <c r="E6" s="10" t="s">
+        <v>39</v>
+      </c>
       <c r="F6" s="1"/>
       <c r="G6" s="1"/>
     </row>
     <row r="7" spans="1:7" ht="21" x14ac:dyDescent="0.35">
-      <c r="A7" s="3"/>
+      <c r="A7" s="18"/>
       <c r="B7" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="C7" s="2"/>
-      <c r="D7" s="2"/>
-      <c r="E7" s="2"/>
+      <c r="C7" s="10" t="s">
+        <v>39</v>
+      </c>
+      <c r="D7" s="10" t="s">
+        <v>39</v>
+      </c>
+      <c r="E7" s="10" t="s">
+        <v>39</v>
+      </c>
       <c r="F7" s="1"/>
       <c r="G7" s="1"/>
     </row>
     <row r="8" spans="1:7" ht="21" x14ac:dyDescent="0.35">
-      <c r="A8" s="4" t="s">
+      <c r="A8" s="11" t="s">
         <v>6</v>
       </c>
-      <c r="B8" s="4" t="s">
+      <c r="B8" s="3" t="s">
         <v>12</v>
       </c>
-      <c r="C8" s="4"/>
-      <c r="D8" s="4"/>
-      <c r="E8" s="4"/>
+      <c r="C8" s="11" t="s">
+        <v>39</v>
+      </c>
+      <c r="D8" s="11" t="s">
+        <v>39</v>
+      </c>
+      <c r="E8" s="11"/>
       <c r="F8" s="1"/>
       <c r="G8" s="1"/>
     </row>
     <row r="9" spans="1:7" ht="21" x14ac:dyDescent="0.35">
-      <c r="A9" s="4"/>
-      <c r="B9" s="4" t="s">
+      <c r="A9" s="11"/>
+      <c r="B9" s="3" t="s">
         <v>13</v>
       </c>
-      <c r="C9" s="4"/>
-      <c r="D9" s="4"/>
-      <c r="E9" s="4"/>
+      <c r="C9" s="11" t="s">
+        <v>39</v>
+      </c>
+      <c r="D9" s="11" t="s">
+        <v>39</v>
+      </c>
+      <c r="E9" s="11"/>
       <c r="F9" s="1"/>
       <c r="G9" s="1"/>
     </row>
     <row r="10" spans="1:7" ht="21" x14ac:dyDescent="0.35">
-      <c r="A10" s="4"/>
-      <c r="B10" s="4" t="s">
+      <c r="A10" s="11"/>
+      <c r="B10" s="3" t="s">
         <v>14</v>
       </c>
-      <c r="C10" s="4"/>
-      <c r="D10" s="4"/>
-      <c r="E10" s="4"/>
+      <c r="C10" s="11" t="s">
+        <v>39</v>
+      </c>
+      <c r="D10" s="11"/>
+      <c r="E10" s="11"/>
       <c r="F10" s="1"/>
       <c r="G10" s="1"/>
     </row>
     <row r="11" spans="1:7" ht="21" x14ac:dyDescent="0.35">
-      <c r="A11" s="4"/>
-      <c r="B11" s="4" t="s">
+      <c r="A11" s="11"/>
+      <c r="B11" s="3" t="s">
         <v>15</v>
       </c>
-      <c r="C11" s="4"/>
-      <c r="D11" s="4"/>
-      <c r="E11" s="4"/>
+      <c r="C11" s="11" t="s">
+        <v>39</v>
+      </c>
+      <c r="D11" s="11" t="s">
+        <v>39</v>
+      </c>
+      <c r="E11" s="11" t="s">
+        <v>39</v>
+      </c>
       <c r="F11" s="1"/>
       <c r="G11" s="1"/>
     </row>
     <row r="12" spans="1:7" ht="21" x14ac:dyDescent="0.35">
-      <c r="A12" s="4"/>
-      <c r="B12" s="4" t="s">
+      <c r="A12" s="11"/>
+      <c r="B12" s="3" t="s">
         <v>16</v>
       </c>
-      <c r="C12" s="4"/>
-      <c r="D12" s="4"/>
-      <c r="E12" s="4"/>
+      <c r="C12" s="11" t="s">
+        <v>39</v>
+      </c>
+      <c r="D12" s="11" t="s">
+        <v>39</v>
+      </c>
+      <c r="E12" s="11" t="s">
+        <v>39</v>
+      </c>
       <c r="F12" s="1"/>
       <c r="G12" s="1"/>
     </row>
     <row r="13" spans="1:7" ht="21" x14ac:dyDescent="0.35">
-      <c r="A13" s="4"/>
-      <c r="B13" s="4" t="s">
+      <c r="A13" s="11"/>
+      <c r="B13" s="3" t="s">
         <v>17</v>
       </c>
-      <c r="C13" s="4"/>
-      <c r="D13" s="4"/>
-      <c r="E13" s="4"/>
+      <c r="C13" s="11" t="s">
+        <v>39</v>
+      </c>
+      <c r="D13" s="11" t="s">
+        <v>39</v>
+      </c>
+      <c r="E13" s="11" t="s">
+        <v>39</v>
+      </c>
       <c r="F13" s="1"/>
       <c r="G13" s="1"/>
     </row>
     <row r="14" spans="1:7" ht="21" x14ac:dyDescent="0.35">
-      <c r="A14" s="5" t="s">
+      <c r="A14" s="12" t="s">
         <v>7</v>
       </c>
-      <c r="B14" s="5" t="s">
+      <c r="B14" s="4" t="s">
         <v>12</v>
       </c>
-      <c r="C14" s="5"/>
-      <c r="D14" s="5"/>
-      <c r="E14" s="5"/>
+      <c r="C14" s="12" t="s">
+        <v>39</v>
+      </c>
+      <c r="D14" s="12" t="s">
+        <v>39</v>
+      </c>
+      <c r="E14" s="12"/>
       <c r="F14" s="1"/>
       <c r="G14" s="1"/>
     </row>
     <row r="15" spans="1:7" ht="21" x14ac:dyDescent="0.35">
-      <c r="A15" s="6"/>
-      <c r="B15" s="5" t="s">
+      <c r="A15" s="19"/>
+      <c r="B15" s="4" t="s">
         <v>13</v>
       </c>
-      <c r="C15" s="5"/>
-      <c r="D15" s="5"/>
-      <c r="E15" s="5"/>
+      <c r="C15" s="12" t="s">
+        <v>39</v>
+      </c>
+      <c r="D15" s="12" t="s">
+        <v>39</v>
+      </c>
+      <c r="E15" s="12"/>
       <c r="F15" s="1"/>
       <c r="G15" s="1"/>
     </row>
     <row r="16" spans="1:7" ht="21" x14ac:dyDescent="0.35">
-      <c r="A16" s="5"/>
-      <c r="B16" s="5" t="s">
+      <c r="A16" s="12"/>
+      <c r="B16" s="4" t="s">
         <v>14</v>
       </c>
-      <c r="C16" s="5"/>
-      <c r="D16" s="5"/>
-      <c r="E16" s="5"/>
+      <c r="C16" s="12" t="s">
+        <v>39</v>
+      </c>
+      <c r="D16" s="12" t="s">
+        <v>39</v>
+      </c>
+      <c r="E16" s="12"/>
       <c r="F16" s="1"/>
       <c r="G16" s="1"/>
     </row>
     <row r="17" spans="1:7" ht="21" x14ac:dyDescent="0.35">
-      <c r="A17" s="5"/>
-      <c r="B17" s="5" t="s">
+      <c r="A17" s="12"/>
+      <c r="B17" s="4" t="s">
         <v>15</v>
       </c>
-      <c r="C17" s="5"/>
-      <c r="D17" s="5"/>
-      <c r="E17" s="5"/>
+      <c r="C17" s="12" t="s">
+        <v>39</v>
+      </c>
+      <c r="D17" s="12" t="s">
+        <v>39</v>
+      </c>
+      <c r="E17" s="12" t="s">
+        <v>39</v>
+      </c>
       <c r="F17" s="1"/>
       <c r="G17" s="1"/>
     </row>
     <row r="18" spans="1:7" ht="21" x14ac:dyDescent="0.35">
-      <c r="A18" s="5"/>
-      <c r="B18" s="5" t="s">
+      <c r="A18" s="12"/>
+      <c r="B18" s="4" t="s">
         <v>16</v>
       </c>
-      <c r="C18" s="5"/>
-      <c r="D18" s="5"/>
-      <c r="E18" s="5"/>
+      <c r="C18" s="12" t="s">
+        <v>39</v>
+      </c>
+      <c r="D18" s="12" t="s">
+        <v>39</v>
+      </c>
+      <c r="E18" s="12"/>
       <c r="F18" s="1"/>
       <c r="G18" s="1"/>
     </row>
     <row r="19" spans="1:7" ht="21" x14ac:dyDescent="0.35">
-      <c r="A19" s="5"/>
-      <c r="B19" s="5" t="s">
+      <c r="A19" s="12"/>
+      <c r="B19" s="4" t="s">
         <v>17</v>
       </c>
-      <c r="C19" s="5"/>
-      <c r="D19" s="5"/>
-      <c r="E19" s="5"/>
+      <c r="C19" s="12" t="s">
+        <v>39</v>
+      </c>
+      <c r="D19" s="12" t="s">
+        <v>39</v>
+      </c>
+      <c r="E19" s="12" t="s">
+        <v>39</v>
+      </c>
       <c r="F19" s="1"/>
       <c r="G19" s="1"/>
     </row>
     <row r="20" spans="1:7" ht="21" x14ac:dyDescent="0.35">
-      <c r="A20" s="7" t="s">
+      <c r="A20" s="13" t="s">
         <v>8</v>
       </c>
-      <c r="B20" s="7" t="s">
+      <c r="B20" s="5" t="s">
         <v>12</v>
       </c>
-      <c r="C20" s="7"/>
-      <c r="D20" s="7"/>
-      <c r="E20" s="7"/>
-      <c r="F20" s="1"/>
+      <c r="C20" s="13" t="s">
+        <v>39</v>
+      </c>
+      <c r="D20" s="13" t="s">
+        <v>41</v>
+      </c>
+      <c r="E20" s="13"/>
+      <c r="F20" s="1" t="s">
+        <v>40</v>
+      </c>
       <c r="G20" s="1"/>
     </row>
     <row r="21" spans="1:7" ht="21" x14ac:dyDescent="0.35">
-      <c r="A21" s="7"/>
-      <c r="B21" s="7" t="s">
+      <c r="A21" s="13"/>
+      <c r="B21" s="5" t="s">
         <v>13</v>
       </c>
-      <c r="C21" s="7"/>
-      <c r="D21" s="7"/>
-      <c r="E21" s="7"/>
+      <c r="C21" s="13" t="s">
+        <v>39</v>
+      </c>
+      <c r="D21" s="13" t="s">
+        <v>39</v>
+      </c>
+      <c r="E21" s="13"/>
       <c r="F21" s="1"/>
       <c r="G21" s="1"/>
     </row>
     <row r="22" spans="1:7" ht="21" x14ac:dyDescent="0.35">
-      <c r="A22" s="7"/>
-      <c r="B22" s="7" t="s">
+      <c r="A22" s="13"/>
+      <c r="B22" s="5" t="s">
         <v>14</v>
       </c>
-      <c r="C22" s="7"/>
-      <c r="D22" s="7"/>
-      <c r="E22" s="7"/>
-      <c r="F22" s="1"/>
+      <c r="C22" s="13" t="s">
+        <v>39</v>
+      </c>
+      <c r="D22" s="13" t="s">
+        <v>41</v>
+      </c>
+      <c r="E22" s="13"/>
+      <c r="F22" s="1" t="s">
+        <v>42</v>
+      </c>
       <c r="G22" s="1"/>
     </row>
     <row r="23" spans="1:7" ht="21" x14ac:dyDescent="0.35">
-      <c r="A23" s="7"/>
-      <c r="B23" s="7" t="s">
+      <c r="A23" s="13"/>
+      <c r="B23" s="5" t="s">
         <v>15</v>
       </c>
-      <c r="C23" s="7"/>
-      <c r="D23" s="7"/>
-      <c r="E23" s="7"/>
+      <c r="C23" s="13" t="s">
+        <v>39</v>
+      </c>
+      <c r="D23" s="13" t="s">
+        <v>39</v>
+      </c>
+      <c r="E23" s="13"/>
       <c r="F23" s="1"/>
       <c r="G23" s="1"/>
     </row>
     <row r="24" spans="1:7" ht="21" x14ac:dyDescent="0.35">
-      <c r="A24" s="7"/>
-      <c r="B24" s="7" t="s">
+      <c r="A24" s="13"/>
+      <c r="B24" s="5" t="s">
         <v>16</v>
       </c>
-      <c r="C24" s="7"/>
-      <c r="D24" s="7"/>
-      <c r="E24" s="7"/>
+      <c r="C24" s="13" t="s">
+        <v>39</v>
+      </c>
+      <c r="D24" s="13" t="s">
+        <v>39</v>
+      </c>
+      <c r="E24" s="13"/>
       <c r="F24" s="1"/>
       <c r="G24" s="1"/>
     </row>
     <row r="25" spans="1:7" ht="21" x14ac:dyDescent="0.35">
-      <c r="A25" s="7"/>
-      <c r="B25" s="7" t="s">
+      <c r="A25" s="13"/>
+      <c r="B25" s="5" t="s">
         <v>17</v>
       </c>
-      <c r="C25" s="7"/>
-      <c r="D25" s="7"/>
-      <c r="E25" s="7"/>
+      <c r="C25" s="13" t="s">
+        <v>39</v>
+      </c>
+      <c r="D25" s="13" t="s">
+        <v>39</v>
+      </c>
+      <c r="E25" s="13"/>
       <c r="F25" s="1"/>
       <c r="G25" s="1"/>
     </row>
     <row r="26" spans="1:7" ht="21" x14ac:dyDescent="0.35">
-      <c r="A26" s="7"/>
-      <c r="B26" s="7" t="s">
+      <c r="A26" s="13"/>
+      <c r="B26" s="5" t="s">
         <v>18</v>
       </c>
-      <c r="C26" s="7"/>
-      <c r="D26" s="7"/>
-      <c r="E26" s="7"/>
+      <c r="C26" s="13" t="s">
+        <v>39</v>
+      </c>
+      <c r="D26" s="13" t="s">
+        <v>39</v>
+      </c>
+      <c r="E26" s="13" t="s">
+        <v>39</v>
+      </c>
       <c r="F26" s="1"/>
       <c r="G26" s="1"/>
     </row>
     <row r="27" spans="1:7" ht="21" x14ac:dyDescent="0.35">
-      <c r="A27" s="8" t="s">
+      <c r="A27" s="14" t="s">
         <v>9</v>
       </c>
-      <c r="B27" s="8" t="s">
+      <c r="B27" s="6" t="s">
         <v>19</v>
       </c>
-      <c r="C27" s="8"/>
-      <c r="D27" s="8"/>
-      <c r="E27" s="8"/>
+      <c r="C27" s="14" t="s">
+        <v>39</v>
+      </c>
+      <c r="D27" s="14" t="s">
+        <v>39</v>
+      </c>
+      <c r="E27" s="14" t="s">
+        <v>39</v>
+      </c>
       <c r="F27" s="1"/>
       <c r="G27" s="1"/>
     </row>
     <row r="28" spans="1:7" ht="21" x14ac:dyDescent="0.35">
-      <c r="A28" s="8"/>
-      <c r="B28" s="8" t="s">
+      <c r="A28" s="14"/>
+      <c r="B28" s="6" t="s">
         <v>20</v>
       </c>
-      <c r="C28" s="8"/>
-      <c r="D28" s="8"/>
-      <c r="E28" s="8"/>
+      <c r="C28" s="14" t="s">
+        <v>39</v>
+      </c>
+      <c r="D28" s="14" t="s">
+        <v>39</v>
+      </c>
+      <c r="E28" s="14" t="s">
+        <v>39</v>
+      </c>
       <c r="F28" s="1"/>
       <c r="G28" s="1"/>
     </row>
     <row r="29" spans="1:7" ht="21" x14ac:dyDescent="0.35">
-      <c r="A29" s="8"/>
-      <c r="B29" s="8" t="s">
+      <c r="A29" s="14"/>
+      <c r="B29" s="6" t="s">
         <v>21</v>
       </c>
-      <c r="C29" s="8"/>
-      <c r="D29" s="8"/>
-      <c r="E29" s="8"/>
+      <c r="C29" s="14" t="s">
+        <v>39</v>
+      </c>
+      <c r="D29" s="14" t="s">
+        <v>39</v>
+      </c>
+      <c r="E29" s="14" t="s">
+        <v>39</v>
+      </c>
       <c r="F29" s="1"/>
       <c r="G29" s="1"/>
     </row>
     <row r="30" spans="1:7" ht="21" x14ac:dyDescent="0.35">
-      <c r="A30" s="8"/>
-      <c r="B30" s="8" t="s">
+      <c r="A30" s="14"/>
+      <c r="B30" s="6" t="s">
         <v>22</v>
       </c>
-      <c r="C30" s="8"/>
-      <c r="D30" s="8"/>
-      <c r="E30" s="8"/>
+      <c r="C30" s="14"/>
+      <c r="D30" s="14"/>
+      <c r="E30" s="14" t="s">
+        <v>39</v>
+      </c>
       <c r="F30" s="1"/>
       <c r="G30" s="1"/>
     </row>
     <row r="31" spans="1:7" ht="21" x14ac:dyDescent="0.35">
-      <c r="A31" s="8"/>
-      <c r="B31" s="8" t="s">
+      <c r="A31" s="14"/>
+      <c r="B31" s="6" t="s">
         <v>23</v>
       </c>
-      <c r="C31" s="8"/>
-      <c r="D31" s="8"/>
-      <c r="E31" s="8"/>
+      <c r="C31" s="14" t="s">
+        <v>39</v>
+      </c>
+      <c r="D31" s="14" t="s">
+        <v>39</v>
+      </c>
+      <c r="E31" s="14"/>
       <c r="F31" s="1"/>
       <c r="G31" s="1"/>
     </row>
     <row r="32" spans="1:7" ht="21" x14ac:dyDescent="0.35">
-      <c r="A32" s="8"/>
-      <c r="B32" s="8" t="s">
+      <c r="A32" s="14"/>
+      <c r="B32" s="6" t="s">
         <v>24</v>
       </c>
-      <c r="C32" s="8"/>
-      <c r="D32" s="8"/>
-      <c r="E32" s="8"/>
+      <c r="C32" s="14" t="s">
+        <v>39</v>
+      </c>
+      <c r="D32" s="14" t="s">
+        <v>39</v>
+      </c>
+      <c r="E32" s="14"/>
       <c r="F32" s="1"/>
       <c r="G32" s="1"/>
     </row>
     <row r="33" spans="1:7" ht="21" x14ac:dyDescent="0.35">
-      <c r="A33" s="8"/>
-      <c r="B33" s="8" t="s">
+      <c r="A33" s="14"/>
+      <c r="B33" s="6" t="s">
         <v>25</v>
       </c>
-      <c r="C33" s="8"/>
-      <c r="D33" s="8"/>
-      <c r="E33" s="8"/>
+      <c r="C33" s="14"/>
+      <c r="D33" s="14"/>
+      <c r="E33" s="14" t="s">
+        <v>39</v>
+      </c>
       <c r="F33" s="1"/>
       <c r="G33" s="1"/>
     </row>
     <row r="34" spans="1:7" ht="21" x14ac:dyDescent="0.35">
-      <c r="A34" s="8"/>
-      <c r="B34" s="8" t="s">
+      <c r="A34" s="14"/>
+      <c r="B34" s="6" t="s">
         <v>26</v>
       </c>
-      <c r="C34" s="8"/>
-      <c r="D34" s="8"/>
-      <c r="E34" s="8"/>
+      <c r="C34" s="14"/>
+      <c r="D34" s="14"/>
+      <c r="E34" s="14"/>
       <c r="F34" s="1"/>
       <c r="G34" s="1"/>
     </row>
     <row r="35" spans="1:7" ht="21" x14ac:dyDescent="0.35">
-      <c r="A35" s="8"/>
-      <c r="B35" s="8" t="s">
+      <c r="A35" s="14"/>
+      <c r="B35" s="6" t="s">
         <v>28</v>
       </c>
-      <c r="C35" s="8"/>
-      <c r="D35" s="8"/>
-      <c r="E35" s="8"/>
+      <c r="C35" s="14"/>
+      <c r="D35" s="14"/>
+      <c r="E35" s="14"/>
       <c r="F35" s="1"/>
       <c r="G35" s="1"/>
     </row>
     <row r="36" spans="1:7" ht="21" x14ac:dyDescent="0.35">
-      <c r="A36" s="8"/>
-      <c r="B36" s="8" t="s">
+      <c r="A36" s="14"/>
+      <c r="B36" s="6" t="s">
         <v>27</v>
       </c>
-      <c r="C36" s="8"/>
-      <c r="D36" s="8"/>
-      <c r="E36" s="8"/>
+      <c r="C36" s="14"/>
+      <c r="D36" s="14"/>
+      <c r="E36" s="14"/>
       <c r="F36" s="1"/>
       <c r="G36" s="1"/>
     </row>
     <row r="37" spans="1:7" ht="21" x14ac:dyDescent="0.35">
-      <c r="A37" s="9"/>
-      <c r="B37" s="8" t="s">
+      <c r="A37" s="20"/>
+      <c r="B37" s="6" t="s">
         <v>29</v>
       </c>
-      <c r="C37" s="8"/>
-      <c r="D37" s="8"/>
-      <c r="E37" s="8"/>
+      <c r="C37" s="14"/>
+      <c r="D37" s="14"/>
+      <c r="E37" s="14"/>
       <c r="F37" s="1"/>
       <c r="G37" s="1"/>
     </row>
     <row r="38" spans="1:7" ht="21" x14ac:dyDescent="0.35">
-      <c r="A38" s="8"/>
-      <c r="B38" s="8" t="s">
+      <c r="A38" s="14"/>
+      <c r="B38" s="6" t="s">
         <v>15</v>
       </c>
-      <c r="C38" s="8"/>
-      <c r="D38" s="8"/>
-      <c r="E38" s="8"/>
+      <c r="C38" s="14"/>
+      <c r="D38" s="14"/>
+      <c r="E38" s="14"/>
       <c r="F38" s="1"/>
       <c r="G38" s="1"/>
     </row>
     <row r="39" spans="1:7" ht="21" x14ac:dyDescent="0.35">
-      <c r="A39" s="10" t="s">
+      <c r="A39" s="15" t="s">
         <v>10</v>
       </c>
-      <c r="B39" s="10" t="s">
+      <c r="B39" s="7" t="s">
         <v>30</v>
       </c>
-      <c r="C39" s="10"/>
-      <c r="D39" s="10"/>
-      <c r="E39" s="10"/>
+      <c r="C39" s="15"/>
+      <c r="D39" s="15"/>
+      <c r="E39" s="15"/>
       <c r="F39" s="1"/>
       <c r="G39" s="1"/>
     </row>
     <row r="40" spans="1:7" ht="21" x14ac:dyDescent="0.35">
-      <c r="A40" s="10"/>
-      <c r="B40" s="10" t="s">
+      <c r="A40" s="15"/>
+      <c r="B40" s="7" t="s">
         <v>31</v>
       </c>
-      <c r="C40" s="10"/>
-      <c r="D40" s="10"/>
-      <c r="E40" s="10"/>
+      <c r="C40" s="15"/>
+      <c r="D40" s="15"/>
+      <c r="E40" s="15"/>
       <c r="F40" s="1"/>
       <c r="G40" s="1"/>
     </row>
     <row r="41" spans="1:7" ht="21" x14ac:dyDescent="0.35">
-      <c r="A41" s="10"/>
-      <c r="B41" s="10" t="s">
+      <c r="A41" s="15"/>
+      <c r="B41" s="7" t="s">
         <v>36</v>
       </c>
-      <c r="C41" s="10"/>
-      <c r="D41" s="10"/>
-      <c r="E41" s="10"/>
+      <c r="C41" s="15"/>
+      <c r="D41" s="15"/>
+      <c r="E41" s="15"/>
       <c r="F41" s="1"/>
       <c r="G41" s="1"/>
     </row>
     <row r="42" spans="1:7" ht="21" x14ac:dyDescent="0.35">
-      <c r="A42" s="10"/>
-      <c r="B42" s="10" t="s">
+      <c r="A42" s="15"/>
+      <c r="B42" s="7" t="s">
         <v>32</v>
       </c>
-      <c r="C42" s="10"/>
-      <c r="D42" s="10"/>
-      <c r="E42" s="10"/>
+      <c r="C42" s="15"/>
+      <c r="D42" s="15"/>
+      <c r="E42" s="15"/>
       <c r="F42" s="1"/>
       <c r="G42" s="1"/>
     </row>
     <row r="43" spans="1:7" ht="21" x14ac:dyDescent="0.35">
-      <c r="A43" s="10"/>
-      <c r="B43" s="10" t="s">
+      <c r="A43" s="15"/>
+      <c r="B43" s="7" t="s">
         <v>33</v>
       </c>
-      <c r="C43" s="10"/>
-      <c r="D43" s="10"/>
-      <c r="E43" s="10"/>
+      <c r="C43" s="15"/>
+      <c r="D43" s="15"/>
+      <c r="E43" s="15"/>
       <c r="F43" s="1"/>
       <c r="G43" s="1"/>
     </row>
     <row r="44" spans="1:7" ht="21" x14ac:dyDescent="0.35">
-      <c r="A44" s="11"/>
-      <c r="B44" s="10" t="s">
+      <c r="A44" s="21"/>
+      <c r="B44" s="7" t="s">
         <v>35</v>
       </c>
-      <c r="C44" s="10"/>
-      <c r="D44" s="10"/>
-      <c r="E44" s="10"/>
+      <c r="C44" s="15"/>
+      <c r="D44" s="15"/>
+      <c r="E44" s="15"/>
       <c r="F44" s="1"/>
       <c r="G44" s="1"/>
     </row>
     <row r="45" spans="1:7" ht="21" x14ac:dyDescent="0.35">
-      <c r="A45" s="10"/>
-      <c r="B45" s="10" t="s">
+      <c r="A45" s="15"/>
+      <c r="B45" s="7" t="s">
         <v>34</v>
       </c>
-      <c r="C45" s="10"/>
-      <c r="D45" s="10"/>
-      <c r="E45" s="10"/>
+      <c r="C45" s="15"/>
+      <c r="D45" s="15"/>
+      <c r="E45" s="15"/>
       <c r="F45" s="1"/>
       <c r="G45" s="1"/>
     </row>
     <row r="46" spans="1:7" ht="21" x14ac:dyDescent="0.35">
-      <c r="A46" s="10"/>
-      <c r="B46" s="10" t="s">
+      <c r="A46" s="15"/>
+      <c r="B46" s="7" t="s">
         <v>37</v>
       </c>
-      <c r="C46" s="10"/>
-      <c r="D46" s="10"/>
-      <c r="E46" s="10"/>
+      <c r="C46" s="15"/>
+      <c r="D46" s="15"/>
+      <c r="E46" s="15"/>
       <c r="F46" s="1"/>
       <c r="G46" s="1"/>
     </row>
     <row r="47" spans="1:7" ht="21" x14ac:dyDescent="0.35">
-      <c r="A47" s="10"/>
-      <c r="B47" s="10" t="s">
+      <c r="A47" s="15"/>
+      <c r="B47" s="7" t="s">
         <v>38</v>
       </c>
-      <c r="C47" s="10"/>
-      <c r="D47" s="10"/>
-      <c r="E47" s="10"/>
+      <c r="C47" s="15"/>
+      <c r="D47" s="15"/>
+      <c r="E47" s="15"/>
       <c r="F47" s="1"/>
       <c r="G47" s="1"/>
     </row>
     <row r="48" spans="1:7" ht="21" x14ac:dyDescent="0.35">
-      <c r="A48" s="12" t="s">
+      <c r="A48" s="16" t="s">
         <v>11</v>
       </c>
-      <c r="B48" s="12" t="s">
+      <c r="B48" s="8" t="s">
         <v>11</v>
       </c>
-      <c r="C48" s="12"/>
-      <c r="D48" s="12"/>
-      <c r="E48" s="12"/>
+      <c r="C48" s="16"/>
+      <c r="D48" s="16"/>
+      <c r="E48" s="16"/>
       <c r="F48" s="1"/>
       <c r="G48" s="1"/>
     </row>
     <row r="49" spans="1:7" ht="21" x14ac:dyDescent="0.35">
-      <c r="A49" s="1"/>
+      <c r="A49" s="9"/>
       <c r="B49" s="1"/>
-      <c r="C49" s="1"/>
-      <c r="D49" s="1"/>
-      <c r="E49" s="1"/>
+      <c r="C49" s="9"/>
+      <c r="D49" s="9"/>
+      <c r="E49" s="9"/>
       <c r="F49" s="1"/>
       <c r="G49" s="1"/>
     </row>

</xml_diff>

<commit_message>
Add cache for permissions
</commit_message>
<xml_diff>
--- a/Permissions.xlsx
+++ b/Permissions.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Erfan\source\repos\LibraryManagementSystem\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FBF5E708-93C7-4A50-8C35-D8D0E760DAFC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3FACDB0F-A232-4277-936A-8D99D73BA268}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-105" yWindow="0" windowWidth="14325" windowHeight="16305" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="133" uniqueCount="43">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="159" uniqueCount="42">
   <si>
     <t>Permissions</t>
   </si>
@@ -126,9 +126,6 @@
     <t>View Fines By User</t>
   </si>
   <si>
-    <t>View Fines By Book</t>
-  </si>
-  <si>
     <t>View Unpaid Fines By User</t>
   </si>
   <si>
@@ -138,9 +135,6 @@
     <t>My Fines</t>
   </si>
   <si>
-    <t>View Unpaid Fines By Book</t>
-  </si>
-  <si>
     <t>History Of Fines</t>
   </si>
   <si>
@@ -154,6 +148,9 @@
   </si>
   <si>
     <t>Librarian can remove only member, but Admin can remove both.</t>
+  </si>
+  <si>
+    <t>OverDue Loans By Book</t>
   </si>
 </sst>
 </file>
@@ -594,7 +591,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:G49"/>
+  <dimension ref="A1:G48"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="21.7109375" style="17" customWidth="1"/>
@@ -631,10 +628,10 @@
         <v>12</v>
       </c>
       <c r="C2" s="10" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="D2" s="10" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="E2" s="10"/>
       <c r="F2" s="1"/>
@@ -646,10 +643,10 @@
         <v>13</v>
       </c>
       <c r="C3" s="10" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="D3" s="10" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="E3" s="10"/>
       <c r="F3" s="1"/>
@@ -661,7 +658,7 @@
         <v>14</v>
       </c>
       <c r="C4" s="10" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="D4" s="10"/>
       <c r="E4" s="10"/>
@@ -674,13 +671,13 @@
         <v>15</v>
       </c>
       <c r="C5" s="10" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="D5" s="10" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="E5" s="10" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="F5" s="1"/>
       <c r="G5" s="1"/>
@@ -691,13 +688,13 @@
         <v>16</v>
       </c>
       <c r="C6" s="10" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="D6" s="10" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="E6" s="10" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="F6" s="1"/>
       <c r="G6" s="1"/>
@@ -708,13 +705,13 @@
         <v>17</v>
       </c>
       <c r="C7" s="10" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="D7" s="10" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="E7" s="10" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="F7" s="1"/>
       <c r="G7" s="1"/>
@@ -727,10 +724,10 @@
         <v>12</v>
       </c>
       <c r="C8" s="11" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="D8" s="11" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="E8" s="11"/>
       <c r="F8" s="1"/>
@@ -742,10 +739,10 @@
         <v>13</v>
       </c>
       <c r="C9" s="11" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="D9" s="11" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="E9" s="11"/>
       <c r="F9" s="1"/>
@@ -757,7 +754,7 @@
         <v>14</v>
       </c>
       <c r="C10" s="11" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="D10" s="11"/>
       <c r="E10" s="11"/>
@@ -770,13 +767,13 @@
         <v>15</v>
       </c>
       <c r="C11" s="11" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="D11" s="11" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="E11" s="11" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="F11" s="1"/>
       <c r="G11" s="1"/>
@@ -787,13 +784,13 @@
         <v>16</v>
       </c>
       <c r="C12" s="11" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="D12" s="11" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="E12" s="11" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="F12" s="1"/>
       <c r="G12" s="1"/>
@@ -804,13 +801,13 @@
         <v>17</v>
       </c>
       <c r="C13" s="11" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="D13" s="11" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="E13" s="11" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="F13" s="1"/>
       <c r="G13" s="1"/>
@@ -823,10 +820,10 @@
         <v>12</v>
       </c>
       <c r="C14" s="12" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="D14" s="12" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="E14" s="12"/>
       <c r="F14" s="1"/>
@@ -838,10 +835,10 @@
         <v>13</v>
       </c>
       <c r="C15" s="12" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="D15" s="12" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="E15" s="12"/>
       <c r="F15" s="1"/>
@@ -853,10 +850,10 @@
         <v>14</v>
       </c>
       <c r="C16" s="12" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="D16" s="12" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="E16" s="12"/>
       <c r="F16" s="1"/>
@@ -868,13 +865,13 @@
         <v>15</v>
       </c>
       <c r="C17" s="12" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="D17" s="12" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="E17" s="12" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="F17" s="1"/>
       <c r="G17" s="1"/>
@@ -885,10 +882,10 @@
         <v>16</v>
       </c>
       <c r="C18" s="12" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="D18" s="12" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="E18" s="12"/>
       <c r="F18" s="1"/>
@@ -900,13 +897,13 @@
         <v>17</v>
       </c>
       <c r="C19" s="12" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="D19" s="12" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="E19" s="12" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="F19" s="1"/>
       <c r="G19" s="1"/>
@@ -919,14 +916,14 @@
         <v>12</v>
       </c>
       <c r="C20" s="13" t="s">
+        <v>37</v>
+      </c>
+      <c r="D20" s="13" t="s">
         <v>39</v>
-      </c>
-      <c r="D20" s="13" t="s">
-        <v>41</v>
       </c>
       <c r="E20" s="13"/>
       <c r="F20" s="1" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="G20" s="1"/>
     </row>
@@ -936,10 +933,10 @@
         <v>13</v>
       </c>
       <c r="C21" s="13" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="D21" s="13" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="E21" s="13"/>
       <c r="F21" s="1"/>
@@ -951,14 +948,14 @@
         <v>14</v>
       </c>
       <c r="C22" s="13" t="s">
+        <v>37</v>
+      </c>
+      <c r="D22" s="13" t="s">
         <v>39</v>
-      </c>
-      <c r="D22" s="13" t="s">
-        <v>41</v>
       </c>
       <c r="E22" s="13"/>
       <c r="F22" s="1" t="s">
-        <v>42</v>
+        <v>40</v>
       </c>
       <c r="G22" s="1"/>
     </row>
@@ -968,10 +965,10 @@
         <v>15</v>
       </c>
       <c r="C23" s="13" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="D23" s="13" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="E23" s="13"/>
       <c r="F23" s="1"/>
@@ -983,10 +980,10 @@
         <v>16</v>
       </c>
       <c r="C24" s="13" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="D24" s="13" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="E24" s="13"/>
       <c r="F24" s="1"/>
@@ -998,10 +995,10 @@
         <v>17</v>
       </c>
       <c r="C25" s="13" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="D25" s="13" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="E25" s="13"/>
       <c r="F25" s="1"/>
@@ -1013,13 +1010,13 @@
         <v>18</v>
       </c>
       <c r="C26" s="13" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="D26" s="13" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="E26" s="13" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="F26" s="1"/>
       <c r="G26" s="1"/>
@@ -1032,13 +1029,13 @@
         <v>19</v>
       </c>
       <c r="C27" s="14" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="D27" s="14" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="E27" s="14" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="F27" s="1"/>
       <c r="G27" s="1"/>
@@ -1049,13 +1046,13 @@
         <v>20</v>
       </c>
       <c r="C28" s="14" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="D28" s="14" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="E28" s="14" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="F28" s="1"/>
       <c r="G28" s="1"/>
@@ -1066,13 +1063,13 @@
         <v>21</v>
       </c>
       <c r="C29" s="14" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="D29" s="14" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="E29" s="14" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="F29" s="1"/>
       <c r="G29" s="1"/>
@@ -1085,7 +1082,7 @@
       <c r="C30" s="14"/>
       <c r="D30" s="14"/>
       <c r="E30" s="14" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="F30" s="1"/>
       <c r="G30" s="1"/>
@@ -1096,10 +1093,10 @@
         <v>23</v>
       </c>
       <c r="C31" s="14" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="D31" s="14" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="E31" s="14"/>
       <c r="F31" s="1"/>
@@ -1111,10 +1108,10 @@
         <v>24</v>
       </c>
       <c r="C32" s="14" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="D32" s="14" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="E32" s="14"/>
       <c r="F32" s="1"/>
@@ -1128,7 +1125,7 @@
       <c r="C33" s="14"/>
       <c r="D33" s="14"/>
       <c r="E33" s="14" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="F33" s="1"/>
       <c r="G33" s="1"/>
@@ -1138,8 +1135,12 @@
       <c r="B34" s="6" t="s">
         <v>26</v>
       </c>
-      <c r="C34" s="14"/>
-      <c r="D34" s="14"/>
+      <c r="C34" s="14" t="s">
+        <v>37</v>
+      </c>
+      <c r="D34" s="14" t="s">
+        <v>37</v>
+      </c>
       <c r="E34" s="14"/>
       <c r="F34" s="1"/>
       <c r="G34" s="1"/>
@@ -1147,10 +1148,14 @@
     <row r="35" spans="1:7" ht="21" x14ac:dyDescent="0.35">
       <c r="A35" s="14"/>
       <c r="B35" s="6" t="s">
-        <v>28</v>
-      </c>
-      <c r="C35" s="14"/>
-      <c r="D35" s="14"/>
+        <v>41</v>
+      </c>
+      <c r="C35" s="14" t="s">
+        <v>37</v>
+      </c>
+      <c r="D35" s="14" t="s">
+        <v>37</v>
+      </c>
       <c r="E35" s="14"/>
       <c r="F35" s="1"/>
       <c r="G35" s="1"/>
@@ -1158,56 +1163,76 @@
     <row r="36" spans="1:7" ht="21" x14ac:dyDescent="0.35">
       <c r="A36" s="14"/>
       <c r="B36" s="6" t="s">
-        <v>27</v>
-      </c>
-      <c r="C36" s="14"/>
-      <c r="D36" s="14"/>
+        <v>28</v>
+      </c>
+      <c r="C36" s="14" t="s">
+        <v>37</v>
+      </c>
+      <c r="D36" s="14" t="s">
+        <v>37</v>
+      </c>
       <c r="E36" s="14"/>
       <c r="F36" s="1"/>
       <c r="G36" s="1"/>
     </row>
     <row r="37" spans="1:7" ht="21" x14ac:dyDescent="0.35">
-      <c r="A37" s="20"/>
+      <c r="A37" s="14"/>
       <c r="B37" s="6" t="s">
-        <v>29</v>
-      </c>
-      <c r="C37" s="14"/>
-      <c r="D37" s="14"/>
+        <v>27</v>
+      </c>
+      <c r="C37" s="14" t="s">
+        <v>37</v>
+      </c>
+      <c r="D37" s="14" t="s">
+        <v>37</v>
+      </c>
       <c r="E37" s="14"/>
       <c r="F37" s="1"/>
       <c r="G37" s="1"/>
     </row>
     <row r="38" spans="1:7" ht="21" x14ac:dyDescent="0.35">
-      <c r="A38" s="14"/>
+      <c r="A38" s="20"/>
       <c r="B38" s="6" t="s">
-        <v>15</v>
-      </c>
-      <c r="C38" s="14"/>
-      <c r="D38" s="14"/>
+        <v>29</v>
+      </c>
+      <c r="C38" s="14" t="s">
+        <v>37</v>
+      </c>
+      <c r="D38" s="14" t="s">
+        <v>37</v>
+      </c>
       <c r="E38" s="14"/>
       <c r="F38" s="1"/>
       <c r="G38" s="1"/>
     </row>
     <row r="39" spans="1:7" ht="21" x14ac:dyDescent="0.35">
-      <c r="A39" s="15" t="s">
-        <v>10</v>
-      </c>
-      <c r="B39" s="7" t="s">
-        <v>30</v>
-      </c>
-      <c r="C39" s="15"/>
-      <c r="D39" s="15"/>
-      <c r="E39" s="15"/>
+      <c r="A39" s="14"/>
+      <c r="B39" s="6" t="s">
+        <v>15</v>
+      </c>
+      <c r="C39" s="14" t="s">
+        <v>37</v>
+      </c>
+      <c r="D39" s="14" t="s">
+        <v>37</v>
+      </c>
+      <c r="E39" s="14"/>
       <c r="F39" s="1"/>
       <c r="G39" s="1"/>
     </row>
     <row r="40" spans="1:7" ht="21" x14ac:dyDescent="0.35">
-      <c r="A40" s="15"/>
+      <c r="A40" s="15" t="s">
+        <v>10</v>
+      </c>
       <c r="B40" s="7" t="s">
-        <v>31</v>
-      </c>
-      <c r="C40" s="15"/>
-      <c r="D40" s="15"/>
+        <v>30</v>
+      </c>
+      <c r="C40" s="15" t="s">
+        <v>37</v>
+      </c>
+      <c r="D40" s="15" t="s">
+        <v>37</v>
+      </c>
       <c r="E40" s="15"/>
       <c r="F40" s="1"/>
       <c r="G40" s="1"/>
@@ -1215,10 +1240,14 @@
     <row r="41" spans="1:7" ht="21" x14ac:dyDescent="0.35">
       <c r="A41" s="15"/>
       <c r="B41" s="7" t="s">
-        <v>36</v>
-      </c>
-      <c r="C41" s="15"/>
-      <c r="D41" s="15"/>
+        <v>31</v>
+      </c>
+      <c r="C41" s="15" t="s">
+        <v>37</v>
+      </c>
+      <c r="D41" s="15" t="s">
+        <v>37</v>
+      </c>
       <c r="E41" s="15"/>
       <c r="F41" s="1"/>
       <c r="G41" s="1"/>
@@ -1226,21 +1255,27 @@
     <row r="42" spans="1:7" ht="21" x14ac:dyDescent="0.35">
       <c r="A42" s="15"/>
       <c r="B42" s="7" t="s">
-        <v>32</v>
+        <v>35</v>
       </c>
       <c r="C42" s="15"/>
       <c r="D42" s="15"/>
-      <c r="E42" s="15"/>
+      <c r="E42" s="15" t="s">
+        <v>37</v>
+      </c>
       <c r="F42" s="1"/>
       <c r="G42" s="1"/>
     </row>
     <row r="43" spans="1:7" ht="21" x14ac:dyDescent="0.35">
       <c r="A43" s="15"/>
       <c r="B43" s="7" t="s">
-        <v>33</v>
-      </c>
-      <c r="C43" s="15"/>
-      <c r="D43" s="15"/>
+        <v>32</v>
+      </c>
+      <c r="C43" s="15" t="s">
+        <v>37</v>
+      </c>
+      <c r="D43" s="15" t="s">
+        <v>37</v>
+      </c>
       <c r="E43" s="15"/>
       <c r="F43" s="1"/>
       <c r="G43" s="1"/>
@@ -1248,21 +1283,27 @@
     <row r="44" spans="1:7" ht="21" x14ac:dyDescent="0.35">
       <c r="A44" s="21"/>
       <c r="B44" s="7" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="C44" s="15"/>
       <c r="D44" s="15"/>
-      <c r="E44" s="15"/>
+      <c r="E44" s="15" t="s">
+        <v>37</v>
+      </c>
       <c r="F44" s="1"/>
       <c r="G44" s="1"/>
     </row>
     <row r="45" spans="1:7" ht="21" x14ac:dyDescent="0.35">
       <c r="A45" s="15"/>
       <c r="B45" s="7" t="s">
-        <v>34</v>
-      </c>
-      <c r="C45" s="15"/>
-      <c r="D45" s="15"/>
+        <v>33</v>
+      </c>
+      <c r="C45" s="15" t="s">
+        <v>37</v>
+      </c>
+      <c r="D45" s="15" t="s">
+        <v>37</v>
+      </c>
       <c r="E45" s="15"/>
       <c r="F45" s="1"/>
       <c r="G45" s="1"/>
@@ -1270,46 +1311,45 @@
     <row r="46" spans="1:7" ht="21" x14ac:dyDescent="0.35">
       <c r="A46" s="15"/>
       <c r="B46" s="7" t="s">
-        <v>37</v>
-      </c>
-      <c r="C46" s="15"/>
-      <c r="D46" s="15"/>
+        <v>36</v>
+      </c>
+      <c r="C46" s="15" t="s">
+        <v>37</v>
+      </c>
+      <c r="D46" s="15" t="s">
+        <v>37</v>
+      </c>
       <c r="E46" s="15"/>
       <c r="F46" s="1"/>
       <c r="G46" s="1"/>
     </row>
     <row r="47" spans="1:7" ht="21" x14ac:dyDescent="0.35">
-      <c r="A47" s="15"/>
-      <c r="B47" s="7" t="s">
-        <v>38</v>
-      </c>
-      <c r="C47" s="15"/>
-      <c r="D47" s="15"/>
-      <c r="E47" s="15"/>
+      <c r="A47" s="16" t="s">
+        <v>11</v>
+      </c>
+      <c r="B47" s="8" t="s">
+        <v>11</v>
+      </c>
+      <c r="C47" s="16" t="s">
+        <v>37</v>
+      </c>
+      <c r="D47" s="16" t="s">
+        <v>37</v>
+      </c>
+      <c r="E47" s="16" t="s">
+        <v>37</v>
+      </c>
       <c r="F47" s="1"/>
       <c r="G47" s="1"/>
     </row>
     <row r="48" spans="1:7" ht="21" x14ac:dyDescent="0.35">
-      <c r="A48" s="16" t="s">
-        <v>11</v>
-      </c>
-      <c r="B48" s="8" t="s">
-        <v>11</v>
-      </c>
-      <c r="C48" s="16"/>
-      <c r="D48" s="16"/>
-      <c r="E48" s="16"/>
+      <c r="A48" s="9"/>
+      <c r="B48" s="1"/>
+      <c r="C48" s="9"/>
+      <c r="D48" s="9"/>
+      <c r="E48" s="9"/>
       <c r="F48" s="1"/>
       <c r="G48" s="1"/>
-    </row>
-    <row r="49" spans="1:7" ht="21" x14ac:dyDescent="0.35">
-      <c r="A49" s="9"/>
-      <c r="B49" s="1"/>
-      <c r="C49" s="9"/>
-      <c r="D49" s="9"/>
-      <c r="E49" s="9"/>
-      <c r="F49" s="1"/>
-      <c r="G49" s="1"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>